<commit_message>
New structure and including Chemical Recycling Sector
</commit_message>
<xml_diff>
--- a/MODEL/SETS_OPENGEM.xlsx
+++ b/MODEL/SETS_OPENGEM.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68163689-FEC5-4FFC-B54A-0D52D6D64EDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="610" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="610" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INDEX" sheetId="33" r:id="rId1"/>
@@ -2669,13 +2669,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:F8"/>
-  <sheetFormatPr defaultColWidth="9.33203125" defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.28515625" defaultRowHeight="10.199999999999999" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="4.5" style="1" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="6" width="9.33203125" style="2"/>
-    <col min="7" max="16384" width="9.33203125" style="1"/>
+    <col min="1" max="1" width="4.42578125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="20.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="6" width="9.28515625" style="2"/>
+    <col min="7" max="16384" width="9.28515625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -2843,12 +2843,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6AAE7177-5A35-4DF2-8CBD-D25EC3AD703D}">
   <dimension ref="B1:C45"/>
-  <sheetFormatPr defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="10.199999999999999" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.5" customWidth="1"/>
-    <col min="3" max="3" width="26.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="10" width="10.83203125" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.42578125" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="10" width="10.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:3" x14ac:dyDescent="0.2">
@@ -3222,12 +3222,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="B1:C118"/>
-  <sheetFormatPr defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="10.199999999999999" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.5" customWidth="1"/>
-    <col min="3" max="3" width="15.5" customWidth="1"/>
-    <col min="4" max="10" width="10.83203125" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.42578125" customWidth="1"/>
+    <col min="3" max="3" width="15.42578125" customWidth="1"/>
+    <col min="4" max="10" width="10.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:3" x14ac:dyDescent="0.2">
@@ -3541,7 +3541,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{749ADD93-37A3-443A-82CB-BD68F51D91D7}">
   <dimension ref="A1:CW47"/>
-  <sheetFormatPr defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="10.199999999999999" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="29" customWidth="1"/>
   </cols>
@@ -17679,9 +17679,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16DB2BD9-4B3B-4368-A2BE-1A00D09D757E}">
   <dimension ref="A1:FG31"/>
-  <sheetFormatPr defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="10.199999999999999" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:163" x14ac:dyDescent="0.2">
@@ -24451,9 +24451,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6204EFC1-CADB-4F7E-9D96-F9A6586281F2}">
   <dimension ref="C2:D3"/>
-  <sheetFormatPr defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="10.199999999999999" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="4" max="4" width="24.1640625" customWidth="1"/>
+    <col min="4" max="4" width="24.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="3:4" x14ac:dyDescent="0.2">
@@ -24480,9 +24480,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCE714E7-CE11-496E-B008-0414D15C2FBB}">
   <dimension ref="C2:D5"/>
-  <sheetFormatPr defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="10.199999999999999" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="4" max="4" width="12.1640625" customWidth="1"/>
+    <col min="4" max="4" width="12.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="3:4" x14ac:dyDescent="0.2">
@@ -24525,9 +24525,9 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9326A444-3434-4071-806D-D8BDD8FB4641}">
   <dimension ref="C2:D5"/>
-  <sheetFormatPr defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="10.199999999999999" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="4" max="4" width="32.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="32.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="3:4" x14ac:dyDescent="0.2">

</xml_diff>